<commit_message>
MAT013 sucesiones + Control 1 MAT060 ejercicios 1
</commit_message>
<xml_diff>
--- a/MAT013/Cronograma_MAT013_2026-1.xlsx
+++ b/MAT013/Cronograma_MAT013_2026-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ehirsh/Github/Clases_USM_2026_1/MAT013'/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ehirsh/Github/Clases_USM_2026_1/MAT013/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017780C2-D904-C04B-9A98-0BD77379D2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E45BE7-2AF7-CF4F-A2C8-883E8E9D3696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="22580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="800" windowWidth="36000" windowHeight="22580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="78">
   <si>
     <t>Semana 6</t>
   </si>
@@ -270,6 +270,9 @@
   </si>
   <si>
     <t>CERTAMEN 3        Temario: Clases  30 a 38</t>
+  </si>
+  <si>
+    <t>solo hice criterio integral</t>
   </si>
 </sst>
 </file>
@@ -1018,6 +1021,9 @@
       <c r="C10" s="5" t="s">
         <v>40</v>
       </c>
+      <c r="D10" s="11" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3">

</xml_diff>